<commit_message>
Updated Regulatory alerts page and added more testimonials in blog
</commit_message>
<xml_diff>
--- a/content/blogs/From_Academicians.xlsx
+++ b/content/blogs/From_Academicians.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t xml:space="preserve">LEXFIN — Blog Page Content</t>
   </si>
@@ -179,6 +179,330 @@
   <si>
     <t xml:space="preserve">Assistant Professor, Faculty of Law, SGT University, Former Law clerk cum Research Associate, Supreme Court of India</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Trust is what makes life easier and worth living. Trust gives birth to love. By trust you make money. And twisting of trust manifests as FRAUD.  Distrusting everyone and everything is a life of hell. In the todays internet webbed world , you never know how close to you the invisible serpent of Fraud might be lurking around. Tread cautiously and be informed is the mantra to tame the beast... 
+Fraud is the intentional act of deception designed to secure unfair or unlawful gain. It involves concealment of facts, or abuse of trust. In the olden days, fraud was committed through direct, face-to-face interactionssuch as forgery, impersonation, and cheating. However, the digital era has introduced cyber frauds as well in the equation. Today, the most dangerous trend is not merely the existence of these two forms but their </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">convergence</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">. The combination of cyber frauds and physical frauds has made it difficult to detect, investigate, and prevent frauds. The convergence frauds play a more deadly financial havocs across the world.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Physical Frauds
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">In physical frauds there is direct interaction with the victims. Their trust is gained and then they are duped of their assets. Physical frauds can take on many forms, for example  
+Social engineering  The fraudsters contact victims over the phone. They can pose as bank staff and request victims for their PINs or cards and then dispatch couriers to pick up the cards. 
+ATM skimming - Fraudsters attach magnetic-stripe skimmers or hidden cameras on ATMs; they can then encode blank cards and withdraw cash. In Delhi/NCR, from 2019 to 2024, multiple cases were reported where ATM theft was perpetrated through skimmers.
+Insider fraud -</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> employees or contracted workers can steal cash or goods from a business. Then can also sell sensitive company information or customer data to rivals or businesses needing data for quick advantage.
+Property Fraud </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">illegal sale or transfer of property is executed by forging documents and signatures.
+Cheque frauds  cheque fraud is committed by faking the signatures.
+Ponzi Schemes  Ponzi schemes promise abnormally high returns, using funds from new investors to pay earlier ones. They often use photos of celebrities or politicians to appear legitimate. Saradha scam (2013) was a multi-crore chit-fund scam that affected lakhs of depositors. 
+Impersonation  Fraudsters can act as officials or police with fake credentials. They coerce law abiding citizens to fall for their threats.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">
+Cyber Frauds
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Cyber frauds are carried out through computers and internet. Due to world wide digital infrastructure, cyber fraud has witnessed exponential growth. Cyber frauds are more devastating in their scale than physical frauds. Some examples of cyber frauds are  
+Phishing, Smishing and Vishing </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">phishing tricks users via emails to commit the fraud. Smishing uses sms for the same purpose and vishing uses voice calls. For example, scammers may send fake QR code, acting to transfer money but actually stealing your PIN.
+Malware  malicious programs are installed on PCs or mobiles to fetch credentials or bypass authority. They can steal banking logins or inject fraudulent transactions.
+Account Hijack </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">the scammer can use stolen credentials to hijack banking accounts, emails or social media accounts. 
+There are many other cyber scams including online identity fraud, ransomware extortion, and fund-transfer frauds etc, making internet a dangerous place to be for gullible innocents.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">
+The Deadly Cocktail: Convergence of Cyber and Physical Frauds
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">The integration of cyber and physical frauds makes frauds more effective and harder to trace. Hybrid frauds follow multi-stage attacks. The typical steps are  
+Step 1: First Access  Scammers use phishing emails, phone scams (vishing), or physical pretexts (impersonation) to obtain user credentials, account info, or system access. For example, a bank employee might be phished into revealing VPN login, or a customer sends account login to a fake website.
+Step 2: Cyber Breach  Using stolen credentials or malware, attackers breach internal networks or online accounts.  
+Step 3: Physical Advantage  Cyber access is turned to physical advantage: fraudsters may program ATM cash-out malware, disable alarms, or siphon payment data.  
+Step 4: The Theft   Finally, the criminals execute the fraud: conducting large ATM withdrawals, draining accounts online, or diverting cargo shipments.  
+Fraud thrives where controls are weak or processes are lax. Rapid digitization (e.g. mobile payments) expands attack surface. People chatting on social networking sites may inadvertently exchange sensitive information without much worry about safety of the network. We may pass on passwords or banking information without realising someone might be tapping or hacking the system. A large number of people use internet but do not have antivirus installed on their systems, especially home users. This makes their computer akin to a house without locks and bolts. Anyone can gain access  and take away what they like  (your passwords, personal information and sensitive banking information) . 
+High-volume periods (holidays) attract thieves, as do cash-heavy channels (gift cards, cashback ATMs). Globalization and e-commerce also aid fraud. The COVID-19 era saw a spike in online fraud, as more transactions moved digital and oversight lagged.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Prevention Controls
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Preventing hybrid frauds requires a multi-layered approach involving individuals, institutions, and the government. At the individual level, people must avoid sharing sensitive information such as OTPs, banking details, or identity documents, even if the request appears to come from trusted authorities. Verifying identities through official channels, rather than relying on phone calls or digital messages, is essential. Financial institutions should adopt advanced technologies like AI-based fraud detection, multi-factor authentication, and real-time transaction monitoring to identify suspicious activities. Regular audits of KYC processes can help prevent misuse of identity documents. Law enforcement agencies must strengthen coordination between cyber cells and traditional policing units to tackle the blended nature of such crimes. Public awareness campaigns, especially in regional languages, can help educate vulnerable populations about evolving fraud tactics like fake investment apps or digital arrest scams. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Conclusion
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Fraudswhether cyber or physicalpose serious threats to individuals and society. While cyber fraud is increasing rapidly due to digitalization, physical fraud continues to exist due to lack of awareness and verification. Both forms of fraud exploit human trust and system vulnerabilities. Prevention of fraud depends on a combination of technological vigilance, legal enforcement, and informed citizen behavior, creating a resilient system against this growing threat. By understanding the nature of these crimes and adopting safe practices, we can protect ourselves and contribute to a more secure society.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms. Uma Devi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistant Professor, IIMT College of Law, Greater Noida </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">In recent years, blockchain and cryptocurrency have become important topics in the world of finance and technology. What started with Bitcoin in 2009 has now developed into a large system that is influencing banking, payments, and investments globally. These technologies are changing how people think about money and financial transactions, especially by reducing dependence on traditional banks and intermediaries.Blockchain is a digital system that records transactions in a secure and transparent manner. Instead of storing data in a single location, it is distributed across multiple computers, making it very difficult to alter or hack. Cryptocurrencies such as Bitcoin and Ethereum are digital currencies that run on this technology and allow people to transfer money directly without the need for banks.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">
+Opportunities of Blockchain and Cryptocurrency
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">One of the biggest advantages of blockchain and cryptocurrency is financial inclusion. Many people around the world still do not have access to banking services. With just a smartphone and internet connection, individuals can send, receive, and store money using cryptocurrencies. This can empower people in rural and underdeveloped areas.Another major benefit is lower transaction cost and faster processing. Traditional financial systems involve multiple intermediaries, which increases both time and cost. Blockchain allows direct peer-to-peer transactions, reducing fees and making international payments much faster.Transparency is also an important feature. Every transaction is recorded on a public ledger, which can be viewed by anyone. This reduces chances of fraud and corruption, especially in areas like supply chains and government transactions.Blockchain has also introduced new financial models like decentralized finance (DeFi). Through DeFi platforms, users can borrow, lend, and invest without banks. Smart contracts automate these processes, reducing the need for manual intervention and making transactions more efficient.Another opportunity is asset tokenization. Real-world assets such as property or stocks can be converted into digital tokens. This allows fractional ownership and makes it easier for people to invest with smaller amounts of money.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Risks and Challenges
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Despite its advantages, blockchain and cryptocurrency also have several risks. One of the biggest issues is price volatility. Cryptocurrency prices can rise or fall rapidly, making them risky for investment and not very stable as a currency.Regulatory uncertainty is another challenge. Different countries have different rules, and many are still developing policies for cryptocurrencies. This creates confusion and risk for investors and businesses.Security is also a concern. While blockchain itself is secure, exchanges and wallets can be hacked. There have been many cases where users lost their funds due to cyberattacks. Also, if someone loses their private key, they permanently lose access to their cryptocurrency.
+Cryptocurrencies can also be misused for illegal activities like money laundering and fraud. Because transactions can be done without full identity verification, it becomes difficult to track users in some cases.Another issue is scalability. Many blockchain networks cannot handle a large number of transactions quickly, leading to delays and higher fees during peak usage.Environmental concerns are also important, especially for cryptocurrencies like Bitcoin that require large amounts of electricity for mining. This has raised questions about sustainability.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Role in Modern Financial Systems
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Blockchain and cryptocurrency are gradually becoming part of modern financial systems. Many banks and financial institutions are exploring blockchain for faster and more secure transactions. It is especially useful in cross-border payments, where traditional systems are slow and expensive.Governments are also working on Central Bank Digital Currencies (CBDCs), which are digital forms of official currency. These aim to combine the benefits of digital payments with government regulation and stability.
+Blockchain is also changing investment and asset management. Tokenization allows assets to be traded digitally, increasing liquidity and making markets more accessible. Financial institutions are also adopting blockchain for record-keeping and fraud detection.At the same time, blockchain is not completely replacing traditional systems but is being integrated with them. This hybrid approach is likely to shape the future of finance.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">
+Conclusion
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Times New Roman"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Blockchain and cryptocurrency have the potential to transform the financial world by making it more efficient, transparent, and inclusive. They provide new opportunities such as low-cost transactions, decentralized finance, and global accessibility. However, they also come with risks like volatility, security issues, and lack of regulation.In the future, the success of these technologies will depend on proper regulation, technological improvements, and wider adoption. If managed correctly, blockchain and cryptocurrency can play a major role in shaping a modern, secure, and inclusive financial system.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms. Shilpi Tyagi </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistant Professor
+At Integrated School of Law, Ghaziabad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National Electronic Funds Transfer (NEFT) and Real Time Gross Settlement (RTGS) are commonly used electronic payment systems in India that allow secure and efficient fund transfers. While these systems are mostly safe, they can be misused if users arent careful.
+One common type of misuse involves fraudsters tricking people into transferring money willingly. Scammers might pretend to be bank officials, employers, or sellers and create a sense of urgency. They might claim theres a problem with your account or offer a deal that seems too good to be true. Once the victim makes a NEFT or RTGS transfer, the transaction is usually irreversible, making it hard to recover the funds.
+Another misuse happens in online marketplace scams. Buyers might be convinced to send advance payments through NEFT or RTGS without checking who they are dealing with. Scammers often vanish after receiving the money, leaving victims facing financial losses.
+Phishing attacks are also a major issue. Users might get fake emails or messages that look like they come from real banks, asking them to confirm account details or approve a transfer. If sensitive information is shared, fraudsters can misuse it to carry out unauthorized transactions.
+To prevent such misuse, its important to follow basic safety practices. Always check the identity of the recipient before sending money. Avoid sharing banking details, OTPs, or passwords with anyone. Be cautious of urgent or emotional requests for money, especially from unknown sources. Additionally, use official banking apps or websites for transactions and keep an eye on your account activity.
+In conclusion, while NEFT and RTGS are trustworthy payment systems, their misuse largely depends on user awareness. Staying informed and alert is essential to protecting your finances.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ms. Diwanshi Rohtagi </t>
+  </si>
 </sst>
 </file>
 
@@ -187,7 +511,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -264,6 +588,39 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="5">
@@ -341,11 +698,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -376,6 +737,22 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -461,9 +838,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1047240</xdr:colOff>
+      <xdr:colOff>1046520</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>1333080</xdr:rowOff>
+      <xdr:rowOff>1332360</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -477,7 +854,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4933800" y="809640"/>
-          <a:ext cx="1047240" cy="1333080"/>
+          <a:ext cx="1046520" cy="1332360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -497,69 +874,114 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="270.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="8" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="1446.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="784.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="309.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>